<commit_message>
automation testing for daraz nepal(login and homepage)
</commit_message>
<xml_diff>
--- a/DarazNP - QA/Daraz_Nepal_QA_TestPlan.xlsx
+++ b/DarazNP - QA/Daraz_Nepal_QA_TestPlan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\QA\DarazNP - QA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DDE6732A-62F1-43A2-A048-E5821CF26FEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43EB3697-1F48-4001-B821-12B2DE4E3B3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" tabRatio="500" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" tabRatio="500" firstSheet="7" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Scenario" sheetId="1" r:id="rId1"/>
@@ -27,12 +27,11 @@
     <sheet name="Summary" sheetId="13" r:id="rId12"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="802" uniqueCount="468">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="467">
   <si>
     <t>Project Name</t>
   </si>
@@ -1277,12 +1276,6 @@
     <t>Tester Name</t>
   </si>
   <si>
-    <t>Test Start Date</t>
-  </si>
-  <si>
-    <t>Test End Date</t>
-  </si>
-  <si>
     <t>Total Test Cases</t>
   </si>
   <si>
@@ -1679,7 +1672,10 @@
     <t>Browser</t>
   </si>
   <si>
-    <t>S</t>
+    <t>Test Start Date(Manual)</t>
+  </si>
+  <si>
+    <t>Test End Date(Manual)</t>
   </si>
 </sst>
 </file>
@@ -1953,21 +1949,6 @@
     <xf numFmtId="14" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1981,6 +1962,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3665,7 +3661,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="C1" s="15"/>
       <c r="D1" s="15"/>
@@ -3685,7 +3681,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C3" s="15"/>
       <c r="D3" s="15"/>
@@ -3722,7 +3718,7 @@
     </row>
     <row r="7" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>9</v>
@@ -3736,7 +3732,7 @@
     </row>
     <row r="8" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="5" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>11</v>
@@ -3750,7 +3746,7 @@
     </row>
     <row r="9" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>12</v>
@@ -3764,7 +3760,7 @@
     </row>
     <row r="10" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="5" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>13</v>
@@ -3778,7 +3774,7 @@
     </row>
     <row r="11" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="5" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>15</v>
@@ -3792,7 +3788,7 @@
     </row>
     <row r="12" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="5" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>17</v>
@@ -3806,7 +3802,7 @@
     </row>
     <row r="13" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="5" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>18</v>
@@ -3820,7 +3816,7 @@
     </row>
     <row r="14" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="5" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>19</v>
@@ -3834,7 +3830,7 @@
     </row>
     <row r="15" spans="1:4" ht="50" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="5" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>20</v>
@@ -3920,7 +3916,7 @@
         <v>32</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>284</v>
@@ -3944,10 +3940,10 @@
         <v>289</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -3955,7 +3951,7 @@
         <v>41</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>290</v>
@@ -3979,10 +3975,10 @@
         <v>295</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -3990,7 +3986,7 @@
         <v>49</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>296</v>
@@ -4014,10 +4010,10 @@
         <v>301</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -4025,7 +4021,7 @@
         <v>56</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>302</v>
@@ -4046,13 +4042,13 @@
         <v>306</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -4060,7 +4056,7 @@
         <v>62</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>307</v>
@@ -4084,10 +4080,10 @@
         <v>313</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -4095,7 +4091,7 @@
         <v>68</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>314</v>
@@ -4119,10 +4115,10 @@
         <v>319</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45"/>
@@ -4208,31 +4204,31 @@
         <v>328</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>360</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>388</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>389</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>362</v>
-      </c>
-      <c r="D2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>390</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="G2" s="5" t="s">
         <v>391</v>
       </c>
-      <c r="F2" s="5" t="s">
-        <v>392</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>393</v>
-      </c>
       <c r="H2" s="5" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="K2" s="5" t="s">
         <v>331</v>
@@ -4244,31 +4240,31 @@
         <v>332</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>392</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>360</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>394</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>362</v>
-      </c>
-      <c r="D3" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>395</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="G3" s="5" t="s">
         <v>396</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>397</v>
       </c>
-      <c r="G3" s="5" t="s">
-        <v>398</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>399</v>
-      </c>
       <c r="I3" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="K3" s="5" t="s">
         <v>331</v>
@@ -4280,31 +4276,31 @@
         <v>333</v>
       </c>
       <c r="B4" s="5" t="s">
+        <v>398</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>362</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>399</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>400</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>364</v>
-      </c>
-      <c r="D4" s="5" t="s">
+      <c r="F4" s="5" t="s">
         <v>401</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="G4" s="5" t="s">
         <v>402</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="H4" s="5" t="s">
         <v>403</v>
       </c>
-      <c r="G4" s="5" t="s">
-        <v>404</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>405</v>
-      </c>
       <c r="I4" s="5" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="K4" s="5" t="s">
         <v>331</v>
@@ -4316,31 +4312,31 @@
         <v>334</v>
       </c>
       <c r="B5" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>356</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>405</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>406</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>358</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>407</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>408</v>
-      </c>
       <c r="F5" s="5" t="s">
+        <v>414</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="H5" s="5" t="s">
         <v>416</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>417</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>418</v>
       </c>
       <c r="I5" s="5" t="s">
         <v>330</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="K5" s="5" t="s">
         <v>331</v>
@@ -4352,28 +4348,28 @@
         <v>335</v>
       </c>
       <c r="B6" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>357</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>409</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>359</v>
-      </c>
-      <c r="D6" s="5" t="s">
+      <c r="F6" s="5" t="s">
         <v>410</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="G6" s="5" t="s">
         <v>411</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="H6" s="5" t="s">
         <v>412</v>
       </c>
-      <c r="G6" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>414</v>
-      </c>
       <c r="I6" s="5" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="J6" s="5" t="s">
         <v>330</v>
@@ -4447,35 +4443,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="23" t="s">
-        <v>388</v>
-      </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
-      <c r="N1" s="23"/>
-      <c r="O1" s="23"/>
+      <c r="A1" s="18" t="s">
+        <v>386</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
+      <c r="M1" s="18"/>
+      <c r="N1" s="18"/>
+      <c r="O1" s="18"/>
     </row>
     <row r="2" spans="1:15" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="3" spans="1:15" ht="21.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A3" s="26" t="s">
-        <v>384</v>
-      </c>
-      <c r="B3" s="26"/>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="26"/>
-      <c r="G3" s="26"/>
+      <c r="A3" s="21" t="s">
+        <v>382</v>
+      </c>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
     </row>
     <row r="4" spans="1:15" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A4" s="4" t="s">
@@ -4518,10 +4514,10 @@
     </row>
     <row r="7" spans="1:15" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A7" s="4" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="C7" s="15"/>
       <c r="D7" s="15"/>
@@ -4534,7 +4530,7 @@
         <v>341</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C8" s="15"/>
       <c r="D8" s="15"/>
@@ -4544,7 +4540,7 @@
     </row>
     <row r="9" spans="1:15" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A9" s="4" t="s">
-        <v>342</v>
+        <v>465</v>
       </c>
       <c r="B9" s="16">
         <v>46163</v>
@@ -4557,9 +4553,11 @@
     </row>
     <row r="10" spans="1:15" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A10" s="4" t="s">
-        <v>343</v>
-      </c>
-      <c r="B10" s="16"/>
+        <v>466</v>
+      </c>
+      <c r="B10" s="16">
+        <v>46166</v>
+      </c>
       <c r="C10" s="15"/>
       <c r="D10" s="15"/>
       <c r="E10" s="15"/>
@@ -4568,170 +4566,167 @@
     </row>
     <row r="11" spans="1:15" ht="18" customHeight="1" thickTop="1" x14ac:dyDescent="0.45"/>
     <row r="12" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A12" s="24" t="s">
+      <c r="A12" s="19" t="s">
+        <v>383</v>
+      </c>
+      <c r="B12" s="19"/>
+      <c r="C12" s="19"/>
+      <c r="E12" s="17" t="s">
         <v>385</v>
       </c>
-      <c r="B12" s="24"/>
-      <c r="C12" s="24"/>
-      <c r="E12" s="22" t="s">
-        <v>387</v>
-      </c>
-      <c r="F12" s="22"/>
-      <c r="G12" s="22"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
     </row>
     <row r="13" spans="1:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="11" t="s">
-        <v>344</v>
-      </c>
-      <c r="B13" s="17">
+        <v>342</v>
+      </c>
+      <c r="B13" s="22">
         <v>56</v>
       </c>
-      <c r="C13" s="17"/>
+      <c r="C13" s="22"/>
       <c r="E13" s="11" t="s">
-        <v>345</v>
-      </c>
-      <c r="F13" s="17">
+        <v>343</v>
+      </c>
+      <c r="F13" s="22">
         <v>5</v>
       </c>
-      <c r="G13" s="17"/>
-      <c r="I13" s="5" t="s">
-        <v>467</v>
-      </c>
+      <c r="G13" s="22"/>
     </row>
     <row r="14" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="11" t="s">
-        <v>346</v>
-      </c>
-      <c r="B14" s="17">
+        <v>344</v>
+      </c>
+      <c r="B14" s="22">
         <v>50</v>
       </c>
-      <c r="C14" s="17"/>
+      <c r="C14" s="22"/>
       <c r="E14" s="11" t="s">
-        <v>347</v>
-      </c>
-      <c r="F14" s="19">
+        <v>345</v>
+      </c>
+      <c r="F14" s="24">
         <v>0</v>
       </c>
-      <c r="G14" s="19"/>
+      <c r="G14" s="24"/>
     </row>
     <row r="15" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="11" t="s">
-        <v>348</v>
-      </c>
-      <c r="B15" s="21">
+        <v>346</v>
+      </c>
+      <c r="B15" s="23">
         <v>49</v>
       </c>
-      <c r="C15" s="21"/>
+      <c r="C15" s="23"/>
       <c r="E15" s="11" t="s">
         <v>330</v>
       </c>
-      <c r="F15" s="19">
+      <c r="F15" s="24">
         <v>1</v>
       </c>
-      <c r="G15" s="19"/>
+      <c r="G15" s="24"/>
     </row>
     <row r="16" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="11" t="s">
-        <v>349</v>
-      </c>
-      <c r="B16" s="19">
+        <v>347</v>
+      </c>
+      <c r="B16" s="24">
         <v>1</v>
       </c>
-      <c r="C16" s="19"/>
+      <c r="C16" s="24"/>
       <c r="E16" s="11" t="s">
-        <v>350</v>
-      </c>
-      <c r="F16" s="20">
+        <v>348</v>
+      </c>
+      <c r="F16" s="26">
         <v>2</v>
       </c>
-      <c r="G16" s="20"/>
+      <c r="G16" s="26"/>
     </row>
     <row r="17" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="11" t="s">
-        <v>351</v>
-      </c>
-      <c r="B17" s="17">
+        <v>349</v>
+      </c>
+      <c r="B17" s="22">
         <v>0</v>
       </c>
-      <c r="C17" s="17"/>
+      <c r="C17" s="22"/>
       <c r="E17" s="11" t="s">
-        <v>352</v>
-      </c>
-      <c r="F17" s="21">
+        <v>350</v>
+      </c>
+      <c r="F17" s="23">
         <v>2</v>
       </c>
-      <c r="G17" s="21"/>
+      <c r="G17" s="23"/>
     </row>
     <row r="18" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="11" t="s">
-        <v>353</v>
-      </c>
-      <c r="B18" s="17">
+        <v>351</v>
+      </c>
+      <c r="B18" s="22">
         <v>0</v>
       </c>
-      <c r="C18" s="17"/>
+      <c r="C18" s="22"/>
       <c r="E18" s="11" t="s">
         <v>331</v>
       </c>
-      <c r="F18" s="17">
+      <c r="F18" s="22">
         <v>5</v>
       </c>
-      <c r="G18" s="17"/>
+      <c r="G18" s="22"/>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="11" t="s">
-        <v>354</v>
-      </c>
-      <c r="B19" s="18">
+        <v>352</v>
+      </c>
+      <c r="B19" s="25">
         <v>0.98</v>
       </c>
-      <c r="C19" s="18"/>
+      <c r="C19" s="25"/>
       <c r="E19" s="11" t="s">
-        <v>355</v>
-      </c>
-      <c r="F19" s="17">
+        <v>353</v>
+      </c>
+      <c r="F19" s="22">
         <v>0</v>
       </c>
-      <c r="G19" s="17"/>
+      <c r="G19" s="22"/>
     </row>
     <row r="20" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="21" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A21" s="25" t="s">
-        <v>386</v>
-      </c>
-      <c r="B21" s="25"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
+      <c r="A21" s="20" t="s">
+        <v>384</v>
+      </c>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20"/>
     </row>
     <row r="22" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="5" t="s">
         <v>322</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="D22" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="E22" s="5" t="s">
         <v>349</v>
       </c>
-      <c r="E22" s="5" t="s">
+      <c r="F22" s="5" t="s">
         <v>351</v>
       </c>
-      <c r="F22" s="5" t="s">
-        <v>353</v>
-      </c>
       <c r="G22" s="5" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="5" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B23" s="5">
         <v>6</v>
@@ -4777,7 +4772,7 @@
     </row>
     <row r="25" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="5" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B25" s="5">
         <v>3</v>
@@ -4800,7 +4795,7 @@
     </row>
     <row r="26" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="5" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B26" s="5">
         <v>4</v>
@@ -4823,7 +4818,7 @@
     </row>
     <row r="27" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="5" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B27" s="5">
         <v>5</v>
@@ -4846,7 +4841,7 @@
     </row>
     <row r="28" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="5" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B28" s="5">
         <v>5</v>
@@ -4869,7 +4864,7 @@
     </row>
     <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="5" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="B29" s="5">
         <v>7</v>
@@ -4892,7 +4887,7 @@
     </row>
     <row r="30" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="5" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B30" s="5">
         <v>5</v>
@@ -4915,7 +4910,7 @@
     </row>
     <row r="31" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="5" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="B31" s="5">
         <v>6</v>
@@ -4940,6 +4935,16 @@
     <row r="33" ht="18" customHeight="1" x14ac:dyDescent="0.45"/>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="F19:G19"/>
     <mergeCell ref="E12:G12"/>
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A12:C12"/>
@@ -4956,16 +4961,6 @@
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="F19:G19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -5057,10 +5052,10 @@
         <v>40</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -5092,10 +5087,10 @@
         <v>48</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -5127,10 +5122,10 @@
         <v>55</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -5162,10 +5157,10 @@
         <v>61</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -5197,10 +5192,10 @@
         <v>67</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -5229,13 +5224,13 @@
         <v>72</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
   </sheetData>
@@ -5316,7 +5311,7 @@
         <v>32</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>73</v>
@@ -5340,10 +5335,10 @@
         <v>79</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -5351,7 +5346,7 @@
         <v>41</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>80</v>
@@ -5375,10 +5370,10 @@
         <v>85</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -5386,7 +5381,7 @@
         <v>49</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>80</v>
@@ -5410,10 +5405,10 @@
         <v>85</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -5421,7 +5416,7 @@
         <v>56</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>80</v>
@@ -5445,10 +5440,10 @@
         <v>85</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -5456,7 +5451,7 @@
         <v>62</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>80</v>
@@ -5480,10 +5475,10 @@
         <v>95</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -5491,7 +5486,7 @@
         <v>68</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>80</v>
@@ -5515,10 +5510,10 @@
         <v>95</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -5526,7 +5521,7 @@
         <v>99</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>80</v>
@@ -5550,10 +5545,10 @@
         <v>95</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -5561,7 +5556,7 @@
         <v>103</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>80</v>
@@ -5585,10 +5580,10 @@
         <v>95</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -5596,7 +5591,7 @@
         <v>107</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>80</v>
@@ -5620,10 +5615,10 @@
         <v>95</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45"/>
@@ -5705,7 +5700,7 @@
         <v>32</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>110</v>
@@ -5729,10 +5724,10 @@
         <v>115</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="57" x14ac:dyDescent="0.45">
@@ -5740,7 +5735,7 @@
         <v>41</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>116</v>
@@ -5764,10 +5759,10 @@
         <v>121</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="57" x14ac:dyDescent="0.45">
@@ -5775,7 +5770,7 @@
         <v>49</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>122</v>
@@ -5799,10 +5794,10 @@
         <v>127</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
   </sheetData>
@@ -5907,10 +5902,10 @@
         <v>135</v>
       </c>
       <c r="J2" s="13" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="K2" s="13" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="42.75" x14ac:dyDescent="0.45">
@@ -5942,10 +5937,10 @@
         <v>142</v>
       </c>
       <c r="J3" s="13" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="K3" s="13" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="42.75" x14ac:dyDescent="0.45">
@@ -5977,10 +5972,10 @@
         <v>146</v>
       </c>
       <c r="J4" s="13" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="K4" s="13" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.45">
@@ -6012,10 +6007,10 @@
         <v>153</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="K5" s="13" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
   </sheetData>
@@ -6119,10 +6114,10 @@
         <v>161</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -6154,10 +6149,10 @@
         <v>167</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -6189,10 +6184,10 @@
         <v>172</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -6224,10 +6219,10 @@
         <v>177</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -6259,10 +6254,10 @@
         <v>182</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
   </sheetData>
@@ -6344,7 +6339,7 @@
         <v>32</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>183</v>
@@ -6368,10 +6363,10 @@
         <v>189</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -6379,7 +6374,7 @@
         <v>41</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>190</v>
@@ -6403,10 +6398,10 @@
         <v>194</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -6414,7 +6409,7 @@
         <v>49</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>190</v>
@@ -6438,10 +6433,10 @@
         <v>199</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -6449,7 +6444,7 @@
         <v>56</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>190</v>
@@ -6473,10 +6468,10 @@
         <v>204</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -6484,7 +6479,7 @@
         <v>62</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>205</v>
@@ -6508,10 +6503,10 @@
         <v>210</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
   </sheetData>
@@ -6602,7 +6597,7 @@
         <v>32</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>211</v>
@@ -6626,10 +6621,10 @@
         <v>216</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="51" customHeight="1" x14ac:dyDescent="0.45">
@@ -6637,7 +6632,7 @@
         <v>41</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>217</v>
@@ -6661,10 +6656,10 @@
         <v>223</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -6672,7 +6667,7 @@
         <v>49</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>224</v>
@@ -6696,10 +6691,10 @@
         <v>230</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -6707,7 +6702,7 @@
         <v>56</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>231</v>
@@ -6731,10 +6726,10 @@
         <v>237</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -6742,7 +6737,7 @@
         <v>62</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>238</v>
@@ -6766,10 +6761,10 @@
         <v>242</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -6777,7 +6772,7 @@
         <v>68</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>243</v>
@@ -6801,10 +6796,10 @@
         <v>247</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -6812,7 +6807,7 @@
         <v>99</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>248</v>
@@ -6836,10 +6831,10 @@
         <v>252</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45"/>
@@ -6922,7 +6917,7 @@
         <v>32</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>253</v>
@@ -6946,10 +6941,10 @@
         <v>258</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="42.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -6957,7 +6952,7 @@
         <v>41</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>259</v>
@@ -6981,10 +6976,10 @@
         <v>264</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -6992,7 +6987,7 @@
         <v>49</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>265</v>
@@ -7016,10 +7011,10 @@
         <v>270</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -7027,7 +7022,7 @@
         <v>56</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>271</v>
@@ -7051,10 +7046,10 @@
         <v>276</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -7062,7 +7057,7 @@
         <v>62</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>277</v>
@@ -7086,10 +7081,10 @@
         <v>283</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="51.75" customHeight="1" x14ac:dyDescent="0.45"/>

</xml_diff>

<commit_message>
QA of Seach and Add to Cart done.
</commit_message>
<xml_diff>
--- a/DarazNP - QA/Daraz_Nepal_QA_TestPlan.xlsx
+++ b/DarazNP - QA/Daraz_Nepal_QA_TestPlan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\QA\DarazNP - QA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43EB3697-1F48-4001-B821-12B2DE4E3B3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B74C9749-543E-4CDF-8E23-6F02B3C549C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" tabRatio="500" firstSheet="7" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1675,7 +1675,7 @@
     <t>Test Start Date(Manual)</t>
   </si>
   <si>
-    <t>Test End Date(Manual)</t>
+    <t>Test End Date</t>
   </si>
 </sst>
 </file>
@@ -1943,10 +1943,19 @@
     <xf numFmtId="0" fontId="5" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="2" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1961,22 +1970,13 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2176,40 +2176,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color rgb="FFBFBFBF"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2307,6 +2273,45 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2907,16 +2912,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
+        <top style="thin">
+          <color rgb="FFBFBFBF"/>
+        </top>
+      </border>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -3238,230 +3238,230 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DF488C28-E294-4FC5-B88E-45C03C2670F4}" name="Table1" displayName="Table1" ref="A6:D15" totalsRowShown="0" headerRowDxfId="150" dataDxfId="149" headerRowCellStyle="Normal" dataCellStyle="Normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DF488C28-E294-4FC5-B88E-45C03C2670F4}" name="Table1" displayName="Table1" ref="A6:D15" totalsRowShown="0" headerRowDxfId="153" dataDxfId="152" headerRowCellStyle="Normal" dataCellStyle="Normal">
   <autoFilter ref="A6:D15" xr:uid="{DF488C28-E294-4FC5-B88E-45C03C2670F4}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{33DAD9C3-616B-4530-8A09-EA2123236523}" name="Test Scenario ID" dataDxfId="148" dataCellStyle="Normal"/>
-    <tableColumn id="2" xr3:uid="{930616D5-B050-48B4-BC07-2F47085FC38F}" name="Test Scenario Description" dataDxfId="147" dataCellStyle="Normal"/>
-    <tableColumn id="3" xr3:uid="{81B53550-0158-483A-8072-7528B8991C66}" name="Priority" dataDxfId="146" dataCellStyle="Normal"/>
-    <tableColumn id="4" xr3:uid="{4E0C06DA-320E-4E35-ABDA-665C29E66893}" name="Number of Test Cases" dataDxfId="145" dataCellStyle="Normal"/>
+    <tableColumn id="1" xr3:uid="{33DAD9C3-616B-4530-8A09-EA2123236523}" name="Test Scenario ID" dataDxfId="151" dataCellStyle="Normal"/>
+    <tableColumn id="2" xr3:uid="{930616D5-B050-48B4-BC07-2F47085FC38F}" name="Test Scenario Description" dataDxfId="150" dataCellStyle="Normal"/>
+    <tableColumn id="3" xr3:uid="{81B53550-0158-483A-8072-7528B8991C66}" name="Priority" dataDxfId="149" dataCellStyle="Normal"/>
+    <tableColumn id="4" xr3:uid="{4E0C06DA-320E-4E35-ABDA-665C29E66893}" name="Number of Test Cases" dataDxfId="148" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{7325E5B5-E902-49F8-AEF5-E792747C2CB9}" name="Table10" displayName="Table10" ref="A1:K7" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{7325E5B5-E902-49F8-AEF5-E792747C2CB9}" name="Table10" displayName="Table10" ref="A1:K7" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42">
   <autoFilter ref="A1:K7" xr:uid="{7325E5B5-E902-49F8-AEF5-E792747C2CB9}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{3E6BAD88-77A0-44B6-9F2B-5FBB3CE091F2}" name="Test Case ID" dataDxfId="51"/>
-    <tableColumn id="2" xr3:uid="{B6334C76-74C3-494E-9AD8-250558808943}" name="Test Scenario" dataDxfId="50"/>
-    <tableColumn id="3" xr3:uid="{C0ABB8E4-BF9C-4E33-B022-CF3A4DE60B64}" name="Test Case Title" dataDxfId="49"/>
-    <tableColumn id="4" xr3:uid="{9B154E74-7F46-4204-9D85-09FD7A515891}" name="Test Description" dataDxfId="48"/>
-    <tableColumn id="5" xr3:uid="{F1A47D99-EDEF-4DEF-9E20-A7FD7E80C2FF}" name="Precondition" dataDxfId="47"/>
-    <tableColumn id="6" xr3:uid="{B6883181-BD4B-46FB-AA46-5EAB92EFDD14}" name="Test Data" dataDxfId="46"/>
-    <tableColumn id="7" xr3:uid="{CDC1D1E1-7F31-4F2F-A9D6-B5BB49DB18D2}" name="Test Step" dataDxfId="45"/>
-    <tableColumn id="8" xr3:uid="{4EC38E01-73BC-4A40-A90C-FBC00297BCCB}" name="Post Condition" dataDxfId="44"/>
-    <tableColumn id="9" xr3:uid="{8B71CA62-1B8D-4F3C-8F1C-80F149DDCD86}" name="Expected Result" dataDxfId="43"/>
-    <tableColumn id="10" xr3:uid="{2758D08A-14A0-421E-93F0-A1D3EED326FD}" name="Actual Result" dataDxfId="42"/>
-    <tableColumn id="11" xr3:uid="{D4909B32-B834-474B-8873-CE83A7F95DED}" name="Status" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{3E6BAD88-77A0-44B6-9F2B-5FBB3CE091F2}" name="Test Case ID" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{B6334C76-74C3-494E-9AD8-250558808943}" name="Test Scenario" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{C0ABB8E4-BF9C-4E33-B022-CF3A4DE60B64}" name="Test Case Title" dataDxfId="39"/>
+    <tableColumn id="4" xr3:uid="{9B154E74-7F46-4204-9D85-09FD7A515891}" name="Test Description" dataDxfId="38"/>
+    <tableColumn id="5" xr3:uid="{F1A47D99-EDEF-4DEF-9E20-A7FD7E80C2FF}" name="Precondition" dataDxfId="37"/>
+    <tableColumn id="6" xr3:uid="{B6883181-BD4B-46FB-AA46-5EAB92EFDD14}" name="Test Data" dataDxfId="36"/>
+    <tableColumn id="7" xr3:uid="{CDC1D1E1-7F31-4F2F-A9D6-B5BB49DB18D2}" name="Test Step" dataDxfId="35"/>
+    <tableColumn id="8" xr3:uid="{4EC38E01-73BC-4A40-A90C-FBC00297BCCB}" name="Post Condition" dataDxfId="34"/>
+    <tableColumn id="9" xr3:uid="{8B71CA62-1B8D-4F3C-8F1C-80F149DDCD86}" name="Expected Result" dataDxfId="33"/>
+    <tableColumn id="10" xr3:uid="{2758D08A-14A0-421E-93F0-A1D3EED326FD}" name="Actual Result" dataDxfId="32"/>
+    <tableColumn id="11" xr3:uid="{D4909B32-B834-474B-8873-CE83A7F95DED}" name="Status" dataDxfId="31"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{074B61AA-834B-4987-8591-EFE949C0CD3E}" name="Table11" displayName="Table11" ref="A1:L6" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{074B61AA-834B-4987-8591-EFE949C0CD3E}" name="Table11" displayName="Table11" ref="A1:L6" totalsRowShown="0" headerRowDxfId="30" dataDxfId="29">
   <autoFilter ref="A1:L6" xr:uid="{074B61AA-834B-4987-8591-EFE949C0CD3E}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{2E0BA05E-6B29-48D5-8C89-726D7682792E}" name="Bug_ID" dataDxfId="38"/>
-    <tableColumn id="2" xr3:uid="{4D01CBE5-0889-4880-92D7-4B66BC182ECB}" name="TC_ID" dataDxfId="37"/>
-    <tableColumn id="3" xr3:uid="{982AC477-4942-498F-B937-BBBFAD3FE9B0}" name="Module" dataDxfId="36"/>
-    <tableColumn id="4" xr3:uid="{45C656C2-F54B-4624-BEE7-F4B8A9A3F7AA}" name="Bug Title" dataDxfId="35"/>
-    <tableColumn id="5" xr3:uid="{5A4A270F-8EE2-456D-8096-C57A552FA8BD}" name="Description" dataDxfId="34"/>
-    <tableColumn id="6" xr3:uid="{5211538C-C43F-4AE0-A40C-4517593D85B8}" name="Steps to Reproduce" dataDxfId="33"/>
-    <tableColumn id="7" xr3:uid="{0D61D290-BC8B-4DAB-B115-362A2EC84928}" name="Expected Result" dataDxfId="32"/>
-    <tableColumn id="8" xr3:uid="{7C9A10CE-DFC8-4284-B52F-67B1076DE1F2}" name="Actual Result" dataDxfId="31"/>
-    <tableColumn id="9" xr3:uid="{A2A09C9A-0EC4-4EEB-8207-4D4AD9E6C2FE}" name="Severity" dataDxfId="30"/>
-    <tableColumn id="10" xr3:uid="{812B3DBC-B5F8-4461-8B42-A270EC894AB1}" name="Priority" dataDxfId="29"/>
-    <tableColumn id="11" xr3:uid="{84506A51-F862-4873-B24D-6E470DF7E85E}" name="Status" dataDxfId="28"/>
-    <tableColumn id="12" xr3:uid="{98CA703C-ECC2-42FB-AB7E-B2461D8721F0}" name="Screenshot/Notes" dataDxfId="27"/>
+    <tableColumn id="1" xr3:uid="{2E0BA05E-6B29-48D5-8C89-726D7682792E}" name="Bug_ID" dataDxfId="28"/>
+    <tableColumn id="2" xr3:uid="{4D01CBE5-0889-4880-92D7-4B66BC182ECB}" name="TC_ID" dataDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{982AC477-4942-498F-B937-BBBFAD3FE9B0}" name="Module" dataDxfId="26"/>
+    <tableColumn id="4" xr3:uid="{45C656C2-F54B-4624-BEE7-F4B8A9A3F7AA}" name="Bug Title" dataDxfId="25"/>
+    <tableColumn id="5" xr3:uid="{5A4A270F-8EE2-456D-8096-C57A552FA8BD}" name="Description" dataDxfId="24"/>
+    <tableColumn id="6" xr3:uid="{5211538C-C43F-4AE0-A40C-4517593D85B8}" name="Steps to Reproduce" dataDxfId="23"/>
+    <tableColumn id="7" xr3:uid="{0D61D290-BC8B-4DAB-B115-362A2EC84928}" name="Expected Result" dataDxfId="22"/>
+    <tableColumn id="8" xr3:uid="{7C9A10CE-DFC8-4284-B52F-67B1076DE1F2}" name="Actual Result" dataDxfId="21"/>
+    <tableColumn id="9" xr3:uid="{A2A09C9A-0EC4-4EEB-8207-4D4AD9E6C2FE}" name="Severity" dataDxfId="20"/>
+    <tableColumn id="10" xr3:uid="{812B3DBC-B5F8-4461-8B42-A270EC894AB1}" name="Priority" dataDxfId="19"/>
+    <tableColumn id="11" xr3:uid="{84506A51-F862-4873-B24D-6E470DF7E85E}" name="Status" dataDxfId="18"/>
+    <tableColumn id="12" xr3:uid="{98CA703C-ECC2-42FB-AB7E-B2461D8721F0}" name="Screenshot/Notes" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{B5F3787F-2FE5-47F0-A53F-BE14C9EDF880}" name="Table12" displayName="Table12" ref="A22:G31" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25" tableBorderDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{B5F3787F-2FE5-47F0-A53F-BE14C9EDF880}" name="Table12" displayName="Table12" ref="A22:G31" totalsRowShown="0" headerRowDxfId="163" dataDxfId="162" tableBorderDxfId="161">
   <autoFilter ref="A22:G31" xr:uid="{B5F3787F-2FE5-47F0-A53F-BE14C9EDF880}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{9F53F743-51DF-481F-9F33-6444B7379A49}" name="Module" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{8809AAEF-A8F9-436C-8EB8-D71DC356BE56}" name="Total TCs" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{938B6847-EE17-4CDD-B2A0-CF0886EE64B8}" name="Pass" dataDxfId="21"/>
-    <tableColumn id="4" xr3:uid="{4F4A2014-C80D-4909-AADC-157B9CB87F8F}" name="Fail" dataDxfId="20"/>
-    <tableColumn id="5" xr3:uid="{BE788EF4-5FDE-4EB6-B750-431A6DA3708D}" name="Blocked" dataDxfId="19"/>
-    <tableColumn id="6" xr3:uid="{56E5F7D1-FE02-40AD-8B69-C21E5C9D2099}" name="Not Executed" dataDxfId="18"/>
-    <tableColumn id="7" xr3:uid="{0EEA2BFA-1D98-4AB4-9C6E-502E972DD0F6}" name="Pass Rate" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{9F53F743-51DF-481F-9F33-6444B7379A49}" name="Module" dataDxfId="160"/>
+    <tableColumn id="2" xr3:uid="{8809AAEF-A8F9-436C-8EB8-D71DC356BE56}" name="Total TCs" dataDxfId="159"/>
+    <tableColumn id="3" xr3:uid="{938B6847-EE17-4CDD-B2A0-CF0886EE64B8}" name="Pass" dataDxfId="158"/>
+    <tableColumn id="4" xr3:uid="{4F4A2014-C80D-4909-AADC-157B9CB87F8F}" name="Fail" dataDxfId="157"/>
+    <tableColumn id="5" xr3:uid="{BE788EF4-5FDE-4EB6-B750-431A6DA3708D}" name="Blocked" dataDxfId="156"/>
+    <tableColumn id="6" xr3:uid="{56E5F7D1-FE02-40AD-8B69-C21E5C9D2099}" name="Not Executed" dataDxfId="155"/>
+    <tableColumn id="7" xr3:uid="{0EEA2BFA-1D98-4AB4-9C6E-502E972DD0F6}" name="Pass Rate" dataDxfId="154"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4D72BE03-3C67-483F-A000-0CB99AE08007}" name="Table2" displayName="Table2" ref="A1:K7" totalsRowShown="0" headerRowDxfId="144" dataDxfId="143">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4D72BE03-3C67-483F-A000-0CB99AE08007}" name="Table2" displayName="Table2" ref="A1:K7" totalsRowShown="0" headerRowDxfId="147" dataDxfId="146">
   <autoFilter ref="A1:K7" xr:uid="{4D72BE03-3C67-483F-A000-0CB99AE08007}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{DC300589-A232-46E8-8D34-43EA76119908}" name="Test Case ID" dataDxfId="142"/>
-    <tableColumn id="2" xr3:uid="{96321DA6-69B9-4285-96FB-F624E3C3A963}" name="Test Scenario" dataDxfId="141"/>
-    <tableColumn id="3" xr3:uid="{47B1BA56-1BCF-45B6-B32B-B5379B2C21C2}" name="Test Case Title" dataDxfId="140"/>
-    <tableColumn id="4" xr3:uid="{C36FE4A9-C732-4047-A84B-CBFDF06E1798}" name="Test Description" dataDxfId="139"/>
-    <tableColumn id="5" xr3:uid="{D1518DD6-352E-4530-B986-D864E93A5AC8}" name="Precondition" dataDxfId="138"/>
-    <tableColumn id="6" xr3:uid="{8B4D31E2-8543-4172-9800-778AC567D164}" name="Test Data" dataDxfId="137"/>
-    <tableColumn id="7" xr3:uid="{CDA134EC-16A7-4594-9E02-221402834F08}" name="Test Step" dataDxfId="136"/>
-    <tableColumn id="8" xr3:uid="{1B527B44-6496-4F0D-A56D-4413FF4DDDA2}" name="Post Condition" dataDxfId="135"/>
-    <tableColumn id="9" xr3:uid="{B9389CBA-79E5-4A58-9516-26D20F6CBA6E}" name="Expected Result" dataDxfId="134"/>
-    <tableColumn id="10" xr3:uid="{52125505-5EBF-4612-93D2-682D2A1590E0}" name="Actual Result" dataDxfId="133"/>
-    <tableColumn id="11" xr3:uid="{169FE3A8-8576-4034-B520-E3C132891BF5}" name="Status" dataDxfId="132"/>
+    <tableColumn id="1" xr3:uid="{DC300589-A232-46E8-8D34-43EA76119908}" name="Test Case ID" dataDxfId="145"/>
+    <tableColumn id="2" xr3:uid="{96321DA6-69B9-4285-96FB-F624E3C3A963}" name="Test Scenario" dataDxfId="144"/>
+    <tableColumn id="3" xr3:uid="{47B1BA56-1BCF-45B6-B32B-B5379B2C21C2}" name="Test Case Title" dataDxfId="143"/>
+    <tableColumn id="4" xr3:uid="{C36FE4A9-C732-4047-A84B-CBFDF06E1798}" name="Test Description" dataDxfId="142"/>
+    <tableColumn id="5" xr3:uid="{D1518DD6-352E-4530-B986-D864E93A5AC8}" name="Precondition" dataDxfId="141"/>
+    <tableColumn id="6" xr3:uid="{8B4D31E2-8543-4172-9800-778AC567D164}" name="Test Data" dataDxfId="140"/>
+    <tableColumn id="7" xr3:uid="{CDA134EC-16A7-4594-9E02-221402834F08}" name="Test Step" dataDxfId="139"/>
+    <tableColumn id="8" xr3:uid="{1B527B44-6496-4F0D-A56D-4413FF4DDDA2}" name="Post Condition" dataDxfId="138"/>
+    <tableColumn id="9" xr3:uid="{B9389CBA-79E5-4A58-9516-26D20F6CBA6E}" name="Expected Result" dataDxfId="137"/>
+    <tableColumn id="10" xr3:uid="{52125505-5EBF-4612-93D2-682D2A1590E0}" name="Actual Result" dataDxfId="136"/>
+    <tableColumn id="11" xr3:uid="{169FE3A8-8576-4034-B520-E3C132891BF5}" name="Status" dataDxfId="135"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{485A2C55-6434-4192-8808-9E3314484566}" name="Table3" displayName="Table3" ref="A1:K10" totalsRowShown="0" headerRowDxfId="131" dataDxfId="130">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{485A2C55-6434-4192-8808-9E3314484566}" name="Table3" displayName="Table3" ref="A1:K10" totalsRowShown="0" headerRowDxfId="134" dataDxfId="133">
   <autoFilter ref="A1:K10" xr:uid="{485A2C55-6434-4192-8808-9E3314484566}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{961A2C21-4B0E-4E55-850D-8F76158E605A}" name="Test Case ID" dataDxfId="129"/>
-    <tableColumn id="2" xr3:uid="{091711FE-D3C8-4930-B519-8CC8A3B55476}" name="Test Scenario" dataDxfId="128"/>
-    <tableColumn id="3" xr3:uid="{88BABBCB-4F52-4C8E-B0AF-A7B1FEA920E1}" name="Test Case Title" dataDxfId="127"/>
-    <tableColumn id="4" xr3:uid="{89C7C9C1-F533-4481-A1AA-3D2ACF79367C}" name="Test Description" dataDxfId="126"/>
-    <tableColumn id="5" xr3:uid="{7E9B2060-966D-4E6E-87D8-0A35654D3D31}" name="Precondition" dataDxfId="125"/>
-    <tableColumn id="6" xr3:uid="{8212B4F5-4682-42D4-98D2-666EB7851034}" name="Test Data" dataDxfId="124"/>
-    <tableColumn id="7" xr3:uid="{C27ADF5D-D13B-4776-B1DB-99BAC727A1EF}" name="Test Step" dataDxfId="123"/>
-    <tableColumn id="8" xr3:uid="{87D91BD6-44DB-42EC-A509-CF909B0841C6}" name="Post Condition" dataDxfId="122"/>
-    <tableColumn id="9" xr3:uid="{CF0F8DF7-50EC-4BF7-9A2B-B588E2C6AD3C}" name="Expected Result" dataDxfId="121"/>
-    <tableColumn id="10" xr3:uid="{28E800BE-C6F2-40A9-92FE-FB97DA376781}" name="Actual Result" dataDxfId="120"/>
-    <tableColumn id="11" xr3:uid="{A019A1D5-1AC2-4238-9C78-8D26EEBABBDD}" name="Status" dataDxfId="119"/>
+    <tableColumn id="1" xr3:uid="{961A2C21-4B0E-4E55-850D-8F76158E605A}" name="Test Case ID" dataDxfId="132"/>
+    <tableColumn id="2" xr3:uid="{091711FE-D3C8-4930-B519-8CC8A3B55476}" name="Test Scenario" dataDxfId="131"/>
+    <tableColumn id="3" xr3:uid="{88BABBCB-4F52-4C8E-B0AF-A7B1FEA920E1}" name="Test Case Title" dataDxfId="130"/>
+    <tableColumn id="4" xr3:uid="{89C7C9C1-F533-4481-A1AA-3D2ACF79367C}" name="Test Description" dataDxfId="129"/>
+    <tableColumn id="5" xr3:uid="{7E9B2060-966D-4E6E-87D8-0A35654D3D31}" name="Precondition" dataDxfId="128"/>
+    <tableColumn id="6" xr3:uid="{8212B4F5-4682-42D4-98D2-666EB7851034}" name="Test Data" dataDxfId="127"/>
+    <tableColumn id="7" xr3:uid="{C27ADF5D-D13B-4776-B1DB-99BAC727A1EF}" name="Test Step" dataDxfId="126"/>
+    <tableColumn id="8" xr3:uid="{87D91BD6-44DB-42EC-A509-CF909B0841C6}" name="Post Condition" dataDxfId="125"/>
+    <tableColumn id="9" xr3:uid="{CF0F8DF7-50EC-4BF7-9A2B-B588E2C6AD3C}" name="Expected Result" dataDxfId="124"/>
+    <tableColumn id="10" xr3:uid="{28E800BE-C6F2-40A9-92FE-FB97DA376781}" name="Actual Result" dataDxfId="123"/>
+    <tableColumn id="11" xr3:uid="{A019A1D5-1AC2-4238-9C78-8D26EEBABBDD}" name="Status" dataDxfId="122"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{CDD8D6C6-33F1-4988-A8DE-6D9CC0E8CF5A}" name="Table4" displayName="Table4" ref="A1:K4" totalsRowShown="0" headerRowDxfId="118" dataDxfId="117">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{CDD8D6C6-33F1-4988-A8DE-6D9CC0E8CF5A}" name="Table4" displayName="Table4" ref="A1:K4" totalsRowShown="0" headerRowDxfId="121" dataDxfId="120">
   <autoFilter ref="A1:K4" xr:uid="{CDD8D6C6-33F1-4988-A8DE-6D9CC0E8CF5A}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{30F17F19-8468-4A66-86EF-0BD83413ACA1}" name="Test Case ID" dataDxfId="116"/>
-    <tableColumn id="2" xr3:uid="{4A6BE90C-FDB5-4937-A0BB-FD1D07A1E264}" name="Test Scenario" dataDxfId="115"/>
-    <tableColumn id="3" xr3:uid="{A81A0D12-E511-4B28-B531-BA483F89581B}" name="Test Case Title" dataDxfId="114"/>
-    <tableColumn id="4" xr3:uid="{53B96AA9-7E95-49E4-A854-6D23E07EB42E}" name="Test Description" dataDxfId="113"/>
-    <tableColumn id="5" xr3:uid="{43B4D6A6-A260-4A56-B9E0-614CAA640920}" name="Precondition" dataDxfId="112"/>
-    <tableColumn id="6" xr3:uid="{125F2F89-B04E-4C4D-B84C-C5971AA23E32}" name="Test Data" dataDxfId="111"/>
-    <tableColumn id="7" xr3:uid="{532C8225-844B-43DE-B1D4-C10DDE0F4A7C}" name="Test Step" dataDxfId="110"/>
-    <tableColumn id="8" xr3:uid="{B349F424-2BCB-47BB-8B8D-7325C04BE2E2}" name="Post Condition" dataDxfId="109"/>
-    <tableColumn id="9" xr3:uid="{74D85BD0-D32D-46A4-9A02-3587A682A2A5}" name="Expected Result" dataDxfId="108"/>
-    <tableColumn id="10" xr3:uid="{16D75875-4017-4E31-BEF6-C8B6145CA67A}" name="Actual Result" dataDxfId="107"/>
-    <tableColumn id="11" xr3:uid="{6B9A5924-AE80-4BC1-AC2A-514E412DBC11}" name="Status" dataDxfId="106"/>
+    <tableColumn id="1" xr3:uid="{30F17F19-8468-4A66-86EF-0BD83413ACA1}" name="Test Case ID" dataDxfId="119"/>
+    <tableColumn id="2" xr3:uid="{4A6BE90C-FDB5-4937-A0BB-FD1D07A1E264}" name="Test Scenario" dataDxfId="118"/>
+    <tableColumn id="3" xr3:uid="{A81A0D12-E511-4B28-B531-BA483F89581B}" name="Test Case Title" dataDxfId="117"/>
+    <tableColumn id="4" xr3:uid="{53B96AA9-7E95-49E4-A854-6D23E07EB42E}" name="Test Description" dataDxfId="116"/>
+    <tableColumn id="5" xr3:uid="{43B4D6A6-A260-4A56-B9E0-614CAA640920}" name="Precondition" dataDxfId="115"/>
+    <tableColumn id="6" xr3:uid="{125F2F89-B04E-4C4D-B84C-C5971AA23E32}" name="Test Data" dataDxfId="114"/>
+    <tableColumn id="7" xr3:uid="{532C8225-844B-43DE-B1D4-C10DDE0F4A7C}" name="Test Step" dataDxfId="113"/>
+    <tableColumn id="8" xr3:uid="{B349F424-2BCB-47BB-8B8D-7325C04BE2E2}" name="Post Condition" dataDxfId="112"/>
+    <tableColumn id="9" xr3:uid="{74D85BD0-D32D-46A4-9A02-3587A682A2A5}" name="Expected Result" dataDxfId="111"/>
+    <tableColumn id="10" xr3:uid="{16D75875-4017-4E31-BEF6-C8B6145CA67A}" name="Actual Result" dataDxfId="110"/>
+    <tableColumn id="11" xr3:uid="{6B9A5924-AE80-4BC1-AC2A-514E412DBC11}" name="Status" dataDxfId="109"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{2E3F6B91-1F8B-4FE1-A0AC-D1A0FB7AA9CF}" name="Table5" displayName="Table5" ref="A1:K5" totalsRowShown="0" headerRowDxfId="105" dataDxfId="104" tableBorderDxfId="103">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{2E3F6B91-1F8B-4FE1-A0AC-D1A0FB7AA9CF}" name="Table5" displayName="Table5" ref="A1:K5" totalsRowShown="0" headerRowDxfId="108" dataDxfId="107" tableBorderDxfId="106">
   <autoFilter ref="A1:K5" xr:uid="{2E3F6B91-1F8B-4FE1-A0AC-D1A0FB7AA9CF}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{6876B7D9-AED4-40A7-9B3F-EAAE7EC27F19}" name="Test Case ID" dataDxfId="102"/>
-    <tableColumn id="2" xr3:uid="{586F0A72-FB20-402D-B906-57CEC15B5844}" name="Test Scenario" dataDxfId="101"/>
-    <tableColumn id="3" xr3:uid="{FD20C9B8-3526-43CA-8EF7-13306F6F1E73}" name="Test Case Title" dataDxfId="100"/>
-    <tableColumn id="4" xr3:uid="{745A2EB8-ABE5-4979-B5E6-271B46F7EF61}" name="Test Description" dataDxfId="99"/>
-    <tableColumn id="5" xr3:uid="{32B27CD7-3A6A-4BC6-864D-23319902CC30}" name="Precondition" dataDxfId="98"/>
-    <tableColumn id="6" xr3:uid="{3B781098-E0A9-48D9-B5BC-2FB2A26565E5}" name="Test Data" dataDxfId="97"/>
-    <tableColumn id="7" xr3:uid="{45BBE8D4-63E2-416F-ACC2-7CD2C1C91220}" name="Test Step" dataDxfId="96"/>
-    <tableColumn id="8" xr3:uid="{CA3B1689-8E28-4BD5-9C34-18D7D98C1AAC}" name="Post Condition" dataDxfId="95"/>
-    <tableColumn id="9" xr3:uid="{B4CDF521-EE6D-4DF0-872E-9D72AC1E8555}" name="Expected Result" dataDxfId="94"/>
-    <tableColumn id="10" xr3:uid="{E6AAEB15-C80D-4145-B1B3-C95E2ACCF6EF}" name="Actual Result" dataDxfId="93"/>
-    <tableColumn id="11" xr3:uid="{73F576F5-8370-4E97-BEBB-223ABB9B606A}" name="Status" dataDxfId="92"/>
+    <tableColumn id="1" xr3:uid="{6876B7D9-AED4-40A7-9B3F-EAAE7EC27F19}" name="Test Case ID" dataDxfId="105"/>
+    <tableColumn id="2" xr3:uid="{586F0A72-FB20-402D-B906-57CEC15B5844}" name="Test Scenario" dataDxfId="104"/>
+    <tableColumn id="3" xr3:uid="{FD20C9B8-3526-43CA-8EF7-13306F6F1E73}" name="Test Case Title" dataDxfId="103"/>
+    <tableColumn id="4" xr3:uid="{745A2EB8-ABE5-4979-B5E6-271B46F7EF61}" name="Test Description" dataDxfId="102"/>
+    <tableColumn id="5" xr3:uid="{32B27CD7-3A6A-4BC6-864D-23319902CC30}" name="Precondition" dataDxfId="101"/>
+    <tableColumn id="6" xr3:uid="{3B781098-E0A9-48D9-B5BC-2FB2A26565E5}" name="Test Data" dataDxfId="100"/>
+    <tableColumn id="7" xr3:uid="{45BBE8D4-63E2-416F-ACC2-7CD2C1C91220}" name="Test Step" dataDxfId="99"/>
+    <tableColumn id="8" xr3:uid="{CA3B1689-8E28-4BD5-9C34-18D7D98C1AAC}" name="Post Condition" dataDxfId="98"/>
+    <tableColumn id="9" xr3:uid="{B4CDF521-EE6D-4DF0-872E-9D72AC1E8555}" name="Expected Result" dataDxfId="97"/>
+    <tableColumn id="10" xr3:uid="{E6AAEB15-C80D-4145-B1B3-C95E2ACCF6EF}" name="Actual Result" dataDxfId="96"/>
+    <tableColumn id="11" xr3:uid="{73F576F5-8370-4E97-BEBB-223ABB9B606A}" name="Status" dataDxfId="95"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{C4579C64-BF71-4412-B0D5-57B184F01462}" name="Table6" displayName="Table6" ref="A1:K6" totalsRowShown="0" headerRowDxfId="91" dataDxfId="90">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{C4579C64-BF71-4412-B0D5-57B184F01462}" name="Table6" displayName="Table6" ref="A1:K6" totalsRowShown="0" headerRowDxfId="94" dataDxfId="93">
   <autoFilter ref="A1:K6" xr:uid="{C4579C64-BF71-4412-B0D5-57B184F01462}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{0CBAA722-80DA-4B08-85C0-C0643AD8A54D}" name="Test Case ID" dataDxfId="89"/>
-    <tableColumn id="2" xr3:uid="{1AE71C13-BF8A-46EB-8744-52C4492B1CA8}" name="Test Scenario" dataDxfId="88"/>
-    <tableColumn id="3" xr3:uid="{DEF6BFB4-FC3B-4290-BB73-914F5D0B138C}" name="Test Case Title" dataDxfId="87"/>
-    <tableColumn id="4" xr3:uid="{046A0014-010C-4B5D-BF73-3F6A7EA80901}" name="Test Description" dataDxfId="86"/>
-    <tableColumn id="5" xr3:uid="{B0659832-BE71-4176-9A59-0F58481951A5}" name="Precondition" dataDxfId="85"/>
-    <tableColumn id="6" xr3:uid="{86937CF6-785A-4BD5-9949-C42326EF2091}" name="Test Data" dataDxfId="84"/>
-    <tableColumn id="7" xr3:uid="{F4174DC9-407D-4FFC-8A52-D9003B91192F}" name="Test Step" dataDxfId="83"/>
-    <tableColumn id="8" xr3:uid="{8E2C6CB3-792C-458C-89B9-86623CAEAEFC}" name="Post Condition" dataDxfId="82"/>
-    <tableColumn id="9" xr3:uid="{15B93BDE-1870-4194-97A8-207E864C076F}" name="Expected Result" dataDxfId="81"/>
-    <tableColumn id="10" xr3:uid="{11F7E854-2EC6-4E5B-9967-97D2AF75D128}" name="Actual Result" dataDxfId="80"/>
-    <tableColumn id="11" xr3:uid="{8CF96C9E-249C-44E9-B980-052118023CDD}" name="Status" dataDxfId="79"/>
+    <tableColumn id="1" xr3:uid="{0CBAA722-80DA-4B08-85C0-C0643AD8A54D}" name="Test Case ID" dataDxfId="92"/>
+    <tableColumn id="2" xr3:uid="{1AE71C13-BF8A-46EB-8744-52C4492B1CA8}" name="Test Scenario" dataDxfId="91"/>
+    <tableColumn id="3" xr3:uid="{DEF6BFB4-FC3B-4290-BB73-914F5D0B138C}" name="Test Case Title" dataDxfId="90"/>
+    <tableColumn id="4" xr3:uid="{046A0014-010C-4B5D-BF73-3F6A7EA80901}" name="Test Description" dataDxfId="89"/>
+    <tableColumn id="5" xr3:uid="{B0659832-BE71-4176-9A59-0F58481951A5}" name="Precondition" dataDxfId="88"/>
+    <tableColumn id="6" xr3:uid="{86937CF6-785A-4BD5-9949-C42326EF2091}" name="Test Data" dataDxfId="87"/>
+    <tableColumn id="7" xr3:uid="{F4174DC9-407D-4FFC-8A52-D9003B91192F}" name="Test Step" dataDxfId="86"/>
+    <tableColumn id="8" xr3:uid="{8E2C6CB3-792C-458C-89B9-86623CAEAEFC}" name="Post Condition" dataDxfId="85"/>
+    <tableColumn id="9" xr3:uid="{15B93BDE-1870-4194-97A8-207E864C076F}" name="Expected Result" dataDxfId="84"/>
+    <tableColumn id="10" xr3:uid="{11F7E854-2EC6-4E5B-9967-97D2AF75D128}" name="Actual Result" dataDxfId="83"/>
+    <tableColumn id="11" xr3:uid="{8CF96C9E-249C-44E9-B980-052118023CDD}" name="Status" dataDxfId="82"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{C5E2AD33-062C-4FF3-97E2-14489F8737F1}" name="Table7" displayName="Table7" ref="A1:K6" totalsRowShown="0" headerRowDxfId="163" dataDxfId="162">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{C5E2AD33-062C-4FF3-97E2-14489F8737F1}" name="Table7" displayName="Table7" ref="A1:K6" totalsRowShown="0" headerRowDxfId="81" dataDxfId="80">
   <autoFilter ref="A1:K6" xr:uid="{C5E2AD33-062C-4FF3-97E2-14489F8737F1}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{CCBD9104-AFBA-47C3-8646-BBD44D55B38B}" name="Test Case ID" dataDxfId="161"/>
-    <tableColumn id="2" xr3:uid="{31C7960A-934A-41FB-B59F-E05141EDD80A}" name="Test Scenario" dataDxfId="160"/>
-    <tableColumn id="3" xr3:uid="{4AEC1D30-8657-40F5-832C-2953CD84B686}" name="Test Case Title" dataDxfId="159"/>
-    <tableColumn id="4" xr3:uid="{0FFF58E0-3C76-4C11-A76F-388626A5967B}" name="Test Description" dataDxfId="158"/>
-    <tableColumn id="5" xr3:uid="{9407EA85-7D2E-4347-B374-302A957DB7C6}" name="Precondition" dataDxfId="157"/>
-    <tableColumn id="6" xr3:uid="{21F6E5C5-88ED-423D-A4A8-0A4611713610}" name="Test Data" dataDxfId="156"/>
-    <tableColumn id="7" xr3:uid="{9F5F42E4-CFB2-4DA8-8C26-83A88E35D7BF}" name="Test Step" dataDxfId="155"/>
-    <tableColumn id="8" xr3:uid="{94D4F544-5CE4-4724-BB7C-0D5E7E5BA04A}" name="Post Condition" dataDxfId="154"/>
-    <tableColumn id="9" xr3:uid="{EC00A77A-F3B3-4584-88AE-EC522129EB55}" name="Expected Result" dataDxfId="153"/>
-    <tableColumn id="10" xr3:uid="{5B0A3255-9926-4CF2-BF04-AA0AB69B800C}" name="Actual Result" dataDxfId="152"/>
-    <tableColumn id="11" xr3:uid="{FAEC2F86-5C61-44B3-9E1A-0EE2E542A7B9}" name="Status" dataDxfId="151"/>
+    <tableColumn id="1" xr3:uid="{CCBD9104-AFBA-47C3-8646-BBD44D55B38B}" name="Test Case ID" dataDxfId="79"/>
+    <tableColumn id="2" xr3:uid="{31C7960A-934A-41FB-B59F-E05141EDD80A}" name="Test Scenario" dataDxfId="78"/>
+    <tableColumn id="3" xr3:uid="{4AEC1D30-8657-40F5-832C-2953CD84B686}" name="Test Case Title" dataDxfId="77"/>
+    <tableColumn id="4" xr3:uid="{0FFF58E0-3C76-4C11-A76F-388626A5967B}" name="Test Description" dataDxfId="76"/>
+    <tableColumn id="5" xr3:uid="{9407EA85-7D2E-4347-B374-302A957DB7C6}" name="Precondition" dataDxfId="75"/>
+    <tableColumn id="6" xr3:uid="{21F6E5C5-88ED-423D-A4A8-0A4611713610}" name="Test Data" dataDxfId="74"/>
+    <tableColumn id="7" xr3:uid="{9F5F42E4-CFB2-4DA8-8C26-83A88E35D7BF}" name="Test Step" dataDxfId="73"/>
+    <tableColumn id="8" xr3:uid="{94D4F544-5CE4-4724-BB7C-0D5E7E5BA04A}" name="Post Condition" dataDxfId="72"/>
+    <tableColumn id="9" xr3:uid="{EC00A77A-F3B3-4584-88AE-EC522129EB55}" name="Expected Result" dataDxfId="71"/>
+    <tableColumn id="10" xr3:uid="{5B0A3255-9926-4CF2-BF04-AA0AB69B800C}" name="Actual Result" dataDxfId="70"/>
+    <tableColumn id="11" xr3:uid="{FAEC2F86-5C61-44B3-9E1A-0EE2E542A7B9}" name="Status" dataDxfId="69"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{76C7F6F1-DEA0-45ED-9527-F69EBF725CC3}" name="Table8" displayName="Table8" ref="A1:K8" totalsRowShown="0" dataDxfId="78">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{76C7F6F1-DEA0-45ED-9527-F69EBF725CC3}" name="Table8" displayName="Table8" ref="A1:K8" totalsRowShown="0" dataDxfId="68">
   <autoFilter ref="A1:K8" xr:uid="{76C7F6F1-DEA0-45ED-9527-F69EBF725CC3}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{78F7358B-BBF5-4E44-95AB-658611EC578F}" name="Test Case ID" dataDxfId="77"/>
-    <tableColumn id="2" xr3:uid="{4C2135E9-2DC4-4097-B4BC-F2C75DD17DC5}" name="Test Scenario" dataDxfId="76"/>
-    <tableColumn id="3" xr3:uid="{6D5B481E-4B3E-4AB4-B904-FBB02F64973F}" name="Test Case Title" dataDxfId="75"/>
-    <tableColumn id="4" xr3:uid="{C798261B-A80F-41B4-B2FF-A03FB57028CA}" name="Test Description" dataDxfId="74"/>
-    <tableColumn id="5" xr3:uid="{B2C9C8E7-63BF-4BD3-AB7C-0B94F88557DC}" name="Precondition" dataDxfId="73"/>
-    <tableColumn id="6" xr3:uid="{3DCB78A0-24D7-4E9E-A397-A7ED87EDB0DC}" name="Test Data" dataDxfId="72"/>
-    <tableColumn id="7" xr3:uid="{7C1F9FC6-BFAA-4E1F-A192-B44375AC929B}" name="Test Step" dataDxfId="71"/>
-    <tableColumn id="8" xr3:uid="{EEE8B405-347E-49F5-B1D8-F91861C4FC16}" name="Post Condition" dataDxfId="70"/>
-    <tableColumn id="9" xr3:uid="{10C2E695-D46A-4680-BE17-45F9AE21F104}" name="Expected Result" dataDxfId="69"/>
-    <tableColumn id="10" xr3:uid="{C6D62D5E-0EAB-47C0-9C55-C96F9AF6647F}" name="Actual Result" dataDxfId="68"/>
-    <tableColumn id="11" xr3:uid="{789CA9A0-3FA3-467F-8F87-FC85389D8700}" name="Status" dataDxfId="67"/>
+    <tableColumn id="1" xr3:uid="{78F7358B-BBF5-4E44-95AB-658611EC578F}" name="Test Case ID" dataDxfId="67"/>
+    <tableColumn id="2" xr3:uid="{4C2135E9-2DC4-4097-B4BC-F2C75DD17DC5}" name="Test Scenario" dataDxfId="66"/>
+    <tableColumn id="3" xr3:uid="{6D5B481E-4B3E-4AB4-B904-FBB02F64973F}" name="Test Case Title" dataDxfId="65"/>
+    <tableColumn id="4" xr3:uid="{C798261B-A80F-41B4-B2FF-A03FB57028CA}" name="Test Description" dataDxfId="64"/>
+    <tableColumn id="5" xr3:uid="{B2C9C8E7-63BF-4BD3-AB7C-0B94F88557DC}" name="Precondition" dataDxfId="63"/>
+    <tableColumn id="6" xr3:uid="{3DCB78A0-24D7-4E9E-A397-A7ED87EDB0DC}" name="Test Data" dataDxfId="62"/>
+    <tableColumn id="7" xr3:uid="{7C1F9FC6-BFAA-4E1F-A192-B44375AC929B}" name="Test Step" dataDxfId="61"/>
+    <tableColumn id="8" xr3:uid="{EEE8B405-347E-49F5-B1D8-F91861C4FC16}" name="Post Condition" dataDxfId="60"/>
+    <tableColumn id="9" xr3:uid="{10C2E695-D46A-4680-BE17-45F9AE21F104}" name="Expected Result" dataDxfId="59"/>
+    <tableColumn id="10" xr3:uid="{C6D62D5E-0EAB-47C0-9C55-C96F9AF6647F}" name="Actual Result" dataDxfId="58"/>
+    <tableColumn id="11" xr3:uid="{789CA9A0-3FA3-467F-8F87-FC85389D8700}" name="Status" dataDxfId="57"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{977FBCCA-BB0D-471A-B840-B1BF610C9A7E}" name="Table9" displayName="Table9" ref="A1:K6" totalsRowShown="0" headerRowDxfId="66" dataDxfId="65">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{977FBCCA-BB0D-471A-B840-B1BF610C9A7E}" name="Table9" displayName="Table9" ref="A1:K6" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
   <autoFilter ref="A1:K6" xr:uid="{977FBCCA-BB0D-471A-B840-B1BF610C9A7E}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{E14DB9FF-88A1-4EE7-B230-D8894A0E1AFB}" name="Test Case ID" dataDxfId="64"/>
-    <tableColumn id="2" xr3:uid="{D4FC117F-56A6-412F-984A-D6DBFC8F6B01}" name="Test Scenario" dataDxfId="63"/>
-    <tableColumn id="3" xr3:uid="{E5DE9E41-179E-45D8-A348-BD490AC75E5D}" name="Test Case Title" dataDxfId="62"/>
-    <tableColumn id="4" xr3:uid="{89C1E1C2-62E8-4407-A716-9188B6576B51}" name="Test Description" dataDxfId="61"/>
-    <tableColumn id="5" xr3:uid="{9FC31264-0A03-44DC-BB14-CE8594D16932}" name="Precondition" dataDxfId="60"/>
-    <tableColumn id="6" xr3:uid="{52040CDD-D184-449A-AA2D-20B3EB5BD5EF}" name="Test Data" dataDxfId="59"/>
-    <tableColumn id="7" xr3:uid="{057CB6AB-A65B-40E5-BF01-A6F370B4BCA2}" name="Test Step" dataDxfId="58"/>
-    <tableColumn id="8" xr3:uid="{0CADDAEE-24CB-4B0B-BD9A-A1895CB19AC7}" name="Post Condition" dataDxfId="57"/>
-    <tableColumn id="9" xr3:uid="{33917D9D-4F6F-4611-9B5E-C61943DC50AE}" name="Expected Result" dataDxfId="56"/>
-    <tableColumn id="10" xr3:uid="{FEFFF501-E422-47CC-ACA8-7793EF2B2B40}" name="Actual Result" dataDxfId="55"/>
-    <tableColumn id="11" xr3:uid="{BAD0A7C4-8AC6-4E11-87E7-837E3A37BD85}" name="Status" dataDxfId="54"/>
+    <tableColumn id="1" xr3:uid="{E14DB9FF-88A1-4EE7-B230-D8894A0E1AFB}" name="Test Case ID" dataDxfId="54"/>
+    <tableColumn id="2" xr3:uid="{D4FC117F-56A6-412F-984A-D6DBFC8F6B01}" name="Test Scenario" dataDxfId="53"/>
+    <tableColumn id="3" xr3:uid="{E5DE9E41-179E-45D8-A348-BD490AC75E5D}" name="Test Case Title" dataDxfId="52"/>
+    <tableColumn id="4" xr3:uid="{89C1E1C2-62E8-4407-A716-9188B6576B51}" name="Test Description" dataDxfId="51"/>
+    <tableColumn id="5" xr3:uid="{9FC31264-0A03-44DC-BB14-CE8594D16932}" name="Precondition" dataDxfId="50"/>
+    <tableColumn id="6" xr3:uid="{52040CDD-D184-449A-AA2D-20B3EB5BD5EF}" name="Test Data" dataDxfId="49"/>
+    <tableColumn id="7" xr3:uid="{057CB6AB-A65B-40E5-BF01-A6F370B4BCA2}" name="Test Step" dataDxfId="48"/>
+    <tableColumn id="8" xr3:uid="{0CADDAEE-24CB-4B0B-BD9A-A1895CB19AC7}" name="Post Condition" dataDxfId="47"/>
+    <tableColumn id="9" xr3:uid="{33917D9D-4F6F-4611-9B5E-C61943DC50AE}" name="Expected Result" dataDxfId="46"/>
+    <tableColumn id="10" xr3:uid="{FEFFF501-E422-47CC-ACA8-7793EF2B2B40}" name="Actual Result" dataDxfId="45"/>
+    <tableColumn id="11" xr3:uid="{BAD0A7C4-8AC6-4E11-87E7-837E3A37BD85}" name="Status" dataDxfId="44"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3660,41 +3660,41 @@
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="24" t="s">
         <v>364</v>
       </c>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
     </row>
     <row r="2" spans="1:4" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
     </row>
     <row r="3" spans="1:4" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="24" t="s">
         <v>365</v>
       </c>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
     </row>
     <row r="4" spans="1:4" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="16">
+      <c r="B4" s="25">
         <v>46163</v>
       </c>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
     </row>
     <row r="5" spans="1:4" ht="18" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
       <c r="A5" s="2"/>
@@ -4443,263 +4443,263 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="21" t="s">
         <v>386</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
+      <c r="O1" s="21"/>
     </row>
     <row r="2" spans="1:15" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="3" spans="1:15" ht="21.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="26" t="s">
         <v>382</v>
       </c>
-      <c r="B3" s="21"/>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
-      <c r="G3" s="21"/>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
     </row>
     <row r="4" spans="1:15" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A4" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="24" t="s">
         <v>336</v>
       </c>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
     </row>
     <row r="5" spans="1:15" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A5" s="4" t="s">
         <v>337</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="24" t="s">
         <v>338</v>
       </c>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
     </row>
     <row r="6" spans="1:15" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A6" s="4" t="s">
         <v>339</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="24" t="s">
         <v>340</v>
       </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
+      <c r="C6" s="24"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="24"/>
     </row>
     <row r="7" spans="1:15" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A7" s="4" t="s">
         <v>464</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="24" t="s">
         <v>463</v>
       </c>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="15"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="24"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="24"/>
     </row>
     <row r="8" spans="1:15" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A8" s="4" t="s">
         <v>341</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="24" t="s">
         <v>365</v>
       </c>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="24"/>
     </row>
     <row r="9" spans="1:15" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A9" s="4" t="s">
         <v>465</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="25">
         <v>46163</v>
       </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="24"/>
     </row>
     <row r="10" spans="1:15" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A10" s="4" t="s">
         <v>466</v>
       </c>
-      <c r="B10" s="16">
-        <v>46166</v>
-      </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
+      <c r="B10" s="25">
+        <v>46170</v>
+      </c>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
     </row>
     <row r="11" spans="1:15" ht="18" customHeight="1" thickTop="1" x14ac:dyDescent="0.45"/>
     <row r="12" spans="1:15" x14ac:dyDescent="0.45">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="22" t="s">
         <v>383</v>
       </c>
-      <c r="B12" s="19"/>
-      <c r="C12" s="19"/>
-      <c r="E12" s="17" t="s">
+      <c r="B12" s="22"/>
+      <c r="C12" s="22"/>
+      <c r="E12" s="20" t="s">
         <v>385</v>
       </c>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="20"/>
     </row>
     <row r="13" spans="1:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="11" t="s">
         <v>342</v>
       </c>
-      <c r="B13" s="22">
+      <c r="B13" s="15">
         <v>56</v>
       </c>
-      <c r="C13" s="22"/>
+      <c r="C13" s="15"/>
       <c r="E13" s="11" t="s">
         <v>343</v>
       </c>
-      <c r="F13" s="22">
+      <c r="F13" s="15">
         <v>5</v>
       </c>
-      <c r="G13" s="22"/>
+      <c r="G13" s="15"/>
     </row>
     <row r="14" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="11" t="s">
         <v>344</v>
       </c>
-      <c r="B14" s="22">
+      <c r="B14" s="15">
         <v>50</v>
       </c>
-      <c r="C14" s="22"/>
+      <c r="C14" s="15"/>
       <c r="E14" s="11" t="s">
         <v>345</v>
       </c>
-      <c r="F14" s="24">
+      <c r="F14" s="17">
         <v>0</v>
       </c>
-      <c r="G14" s="24"/>
+      <c r="G14" s="17"/>
     </row>
     <row r="15" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="11" t="s">
         <v>346</v>
       </c>
-      <c r="B15" s="23">
+      <c r="B15" s="19">
         <v>49</v>
       </c>
-      <c r="C15" s="23"/>
+      <c r="C15" s="19"/>
       <c r="E15" s="11" t="s">
         <v>330</v>
       </c>
-      <c r="F15" s="24">
+      <c r="F15" s="17">
         <v>1</v>
       </c>
-      <c r="G15" s="24"/>
+      <c r="G15" s="17"/>
     </row>
     <row r="16" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="11" t="s">
         <v>347</v>
       </c>
-      <c r="B16" s="24">
+      <c r="B16" s="17">
         <v>1</v>
       </c>
-      <c r="C16" s="24"/>
+      <c r="C16" s="17"/>
       <c r="E16" s="11" t="s">
         <v>348</v>
       </c>
-      <c r="F16" s="26">
+      <c r="F16" s="18">
         <v>2</v>
       </c>
-      <c r="G16" s="26"/>
+      <c r="G16" s="18"/>
     </row>
     <row r="17" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="11" t="s">
         <v>349</v>
       </c>
-      <c r="B17" s="22">
+      <c r="B17" s="15">
         <v>0</v>
       </c>
-      <c r="C17" s="22"/>
+      <c r="C17" s="15"/>
       <c r="E17" s="11" t="s">
         <v>350</v>
       </c>
-      <c r="F17" s="23">
+      <c r="F17" s="19">
         <v>2</v>
       </c>
-      <c r="G17" s="23"/>
+      <c r="G17" s="19"/>
     </row>
     <row r="18" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="11" t="s">
         <v>351</v>
       </c>
-      <c r="B18" s="22">
+      <c r="B18" s="15">
         <v>0</v>
       </c>
-      <c r="C18" s="22"/>
+      <c r="C18" s="15"/>
       <c r="E18" s="11" t="s">
         <v>331</v>
       </c>
-      <c r="F18" s="22">
+      <c r="F18" s="15">
         <v>5</v>
       </c>
-      <c r="G18" s="22"/>
+      <c r="G18" s="15"/>
     </row>
     <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="11" t="s">
         <v>352</v>
       </c>
-      <c r="B19" s="25">
+      <c r="B19" s="16">
         <v>0.98</v>
       </c>
-      <c r="C19" s="25"/>
+      <c r="C19" s="16"/>
       <c r="E19" s="11" t="s">
         <v>353</v>
       </c>
-      <c r="F19" s="22">
+      <c r="F19" s="15">
         <v>0</v>
       </c>
-      <c r="G19" s="22"/>
+      <c r="G19" s="15"/>
     </row>
     <row r="20" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="21" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A21" s="20" t="s">
+      <c r="A21" s="23" t="s">
         <v>384</v>
       </c>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
-      <c r="E21" s="20"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="20"/>
+      <c r="B21" s="23"/>
+      <c r="C21" s="23"/>
+      <c r="D21" s="23"/>
+      <c r="E21" s="23"/>
+      <c r="F21" s="23"/>
+      <c r="G21" s="23"/>
     </row>
     <row r="22" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="5" t="s">
@@ -4935,16 +4935,6 @@
     <row r="33" ht="18" customHeight="1" x14ac:dyDescent="0.45"/>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="F19:G19"/>
     <mergeCell ref="E12:G12"/>
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A12:C12"/>
@@ -4961,6 +4951,16 @@
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="F19:G19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>